<commit_message>
update arch and benefit
</commit_message>
<xml_diff>
--- a/RoadMap.xlsx
+++ b/RoadMap.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0703F9BC-4E1A-4CCA-B8BE-2D3C6F82D133}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29055D71-1B17-400C-B24F-09C3854E97D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Задачи" sheetId="1" r:id="rId1"/>
@@ -185,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -205,6 +205,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -759,7 +762,7 @@
       <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="7" t="s">
         <v>20</v>
       </c>
       <c r="C3" s="4" t="s">
@@ -803,7 +806,7 @@
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
-      <c r="J4" s="2" t="s">
+      <c r="J4" s="8" t="s">
         <v>31</v>
       </c>
     </row>

</xml_diff>